<commit_message>
IKA Update Priority 1 via Panel
</commit_message>
<xml_diff>
--- a/THA(1. ÖNCELİK).xlsx
+++ b/THA(1. ÖNCELİK).xlsx
@@ -520,6 +520,12 @@
       <c r="H4" t="str">
         <v>ÇAVUŞLU-0/1519, ÇAVUŞLU-0/3887, ÇAVUŞLU-0/86, ÇAVUŞLU-0/88, ÇAVUŞLU-9980/1, ÇAVUŞLU-9980/18, ÇAVUŞLU-9981/1, ÇAVUŞLU-9981/2, ÇAVUŞLU-9982/1, ÇAVUŞLU-9982/2, ÇAVUŞLU-9982/3, ÇAVUŞLU-9982/4, ÇAVUŞLU-9982/5, ÇAVUŞLU-9982/6, ÇAVUŞLU-9982/7, ÇAVUŞLU-9983/1, ÇAVUŞLU-9983/18, ÇAVUŞLU-9984/1, ÇAVUŞLU-9985/1, ÇAVUŞLU-9985/2, ÇAVUŞLU-9985/25, ÇAVUŞLU-9985/26, ÇAVUŞLU-9985/27, ÇAVUŞLU-9985/28, ÇAVUŞLU-9985/29, ÇAVUŞLU-9985/3, ÇAVUŞLU-9985/30, ÇAVUŞLU-9985/4, ÇAVUŞLU-9985/5, ÇAVUŞLU-9985/6, ÇAVUŞLU-9985/7, ÇAVUŞLU-9986/1, ÇAVUŞLU-9986/2, ÇAVUŞLU-9986/3, ÇAVUŞLU-9986/4, ÇAVUŞLU-9986/5</v>
       </c>
+      <c r="I4" t="str">
+        <v>Gönderildi</v>
+      </c>
+      <c r="J4" t="str">
+        <v>Evet</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">

</xml_diff>